<commit_message>
posted 213 midterm 2 gradelines and lecture 29 notes
</commit_message>
<xml_diff>
--- a/213_S26/gradelines.xlsx
+++ b/213_S26/gradelines.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="E2" s="4">
         <f>100*(SUM(F5:F15)/COUNT(F5:F15)*0.15 + SUM(F19:F25)/COUNT(F19:F25)*0.1 + SUM(F29:F31)*0.15 + F32*0.3)</f>
-        <v>21.94805195</v>
+        <v>30.25974026</v>
       </c>
     </row>
     <row r="3">
@@ -602,7 +602,7 @@
         <v>20.0</v>
       </c>
       <c r="F8" s="8">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="9">
@@ -618,7 +618,7 @@
         <v>20.0</v>
       </c>
       <c r="F9" s="8">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="10">
@@ -634,7 +634,7 @@
         <v>20.0</v>
       </c>
       <c r="F10" s="8">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="11">
@@ -650,7 +650,7 @@
         <v>20.0</v>
       </c>
       <c r="F11" s="8">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="H11" s="11" t="s">
         <v>20</v>
@@ -697,16 +697,18 @@
       </c>
       <c r="I12" s="12">
         <f>0.93*E16</f>
-        <v>55.8</v>
+        <v>130.2</v>
       </c>
       <c r="J12" s="12">
         <f>0.93*E26</f>
-        <v>22.32</v>
+        <v>44.64</v>
       </c>
       <c r="K12" s="12">
         <v>75.0</v>
       </c>
-      <c r="L12" s="12"/>
+      <c r="L12" s="12">
+        <v>70.0</v>
+      </c>
       <c r="M12" s="8"/>
       <c r="N12" s="12"/>
       <c r="O12" s="12">
@@ -734,16 +736,18 @@
       </c>
       <c r="I13" s="12">
         <f>0.9*E16</f>
-        <v>54</v>
+        <v>126</v>
       </c>
       <c r="J13" s="4">
         <f>0.9*E26</f>
-        <v>21.6</v>
+        <v>43.2</v>
       </c>
       <c r="K13" s="12">
         <v>70.0</v>
       </c>
-      <c r="L13" s="12"/>
+      <c r="L13" s="12">
+        <v>66.0</v>
+      </c>
       <c r="M13" s="8"/>
       <c r="N13" s="12"/>
       <c r="O13" s="12">
@@ -771,16 +775,18 @@
       </c>
       <c r="I14" s="12">
         <f>0.87*E16</f>
-        <v>52.2</v>
+        <v>121.8</v>
       </c>
       <c r="J14" s="4">
         <f>0.87*E26</f>
-        <v>20.88</v>
+        <v>41.76</v>
       </c>
       <c r="K14" s="12">
         <v>65.0</v>
       </c>
-      <c r="L14" s="12"/>
+      <c r="L14" s="12">
+        <v>62.0</v>
+      </c>
       <c r="M14" s="8"/>
       <c r="N14" s="12"/>
       <c r="O14" s="12">
@@ -808,16 +814,18 @@
       </c>
       <c r="I15" s="12">
         <f>0.83*E16</f>
-        <v>49.8</v>
+        <v>116.2</v>
       </c>
       <c r="J15" s="4">
         <f>0.83*E26</f>
-        <v>19.92</v>
+        <v>39.84</v>
       </c>
       <c r="K15" s="12">
         <v>60.0</v>
       </c>
-      <c r="L15" s="12"/>
+      <c r="L15" s="12">
+        <v>58.0</v>
+      </c>
       <c r="M15" s="8"/>
       <c r="N15" s="12"/>
       <c r="O15" s="12">
@@ -838,7 +846,7 @@
       </c>
       <c r="E16" s="8">
         <f>20*MIN(SUM(F5:F15),COUNT(F5:F15)-1)</f>
-        <v>60</v>
+        <v>140</v>
       </c>
       <c r="F16" s="8"/>
       <c r="H16" s="8" t="s">
@@ -846,16 +854,18 @@
       </c>
       <c r="I16" s="12">
         <f>0.8*E16</f>
-        <v>48</v>
+        <v>112</v>
       </c>
       <c r="J16" s="4">
         <f>0.8*E26</f>
-        <v>19.2</v>
+        <v>38.4</v>
       </c>
       <c r="K16" s="12">
         <v>55.0</v>
       </c>
-      <c r="L16" s="12"/>
+      <c r="L16" s="12">
+        <v>54.0</v>
+      </c>
       <c r="M16" s="8"/>
       <c r="N16" s="12"/>
       <c r="O16" s="12">
@@ -874,16 +884,18 @@
       </c>
       <c r="I17" s="4">
         <f>0.77*E16</f>
-        <v>46.2</v>
+        <v>107.8</v>
       </c>
       <c r="J17" s="4">
         <f>0.77*E26</f>
-        <v>18.48</v>
+        <v>36.96</v>
       </c>
       <c r="K17" s="12">
         <v>50.0</v>
       </c>
-      <c r="L17" s="12"/>
+      <c r="L17" s="12">
+        <v>50.0</v>
+      </c>
       <c r="M17" s="8"/>
       <c r="N17" s="12"/>
       <c r="O17" s="12">
@@ -912,16 +924,18 @@
       </c>
       <c r="I18" s="4">
         <f>0.73*E16</f>
-        <v>43.8</v>
+        <v>102.2</v>
       </c>
       <c r="J18" s="4">
         <f>0.73*E26</f>
-        <v>17.52</v>
+        <v>35.04</v>
       </c>
       <c r="K18" s="12">
         <v>44.0</v>
       </c>
-      <c r="L18" s="12"/>
+      <c r="L18" s="12">
+        <v>46.0</v>
+      </c>
       <c r="M18" s="8"/>
       <c r="N18" s="12"/>
       <c r="O18" s="12">
@@ -949,16 +963,18 @@
       </c>
       <c r="I19" s="12">
         <f>0.7*E16</f>
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="J19" s="4">
         <f>0.7*E26</f>
-        <v>16.8</v>
+        <v>33.6</v>
       </c>
       <c r="K19" s="12">
         <v>38.0</v>
       </c>
-      <c r="L19" s="12"/>
+      <c r="L19" s="12">
+        <v>40.0</v>
+      </c>
       <c r="M19" s="8"/>
       <c r="N19" s="12"/>
       <c r="O19" s="12">
@@ -986,16 +1002,18 @@
       </c>
       <c r="I20" s="12">
         <f>0.67*E16</f>
-        <v>40.2</v>
+        <v>93.8</v>
       </c>
       <c r="J20" s="4">
         <f>0.67*E26</f>
-        <v>16.08</v>
+        <v>32.16</v>
       </c>
       <c r="K20" s="12">
         <v>32.0</v>
       </c>
-      <c r="L20" s="12"/>
+      <c r="L20" s="12">
+        <v>34.0</v>
+      </c>
       <c r="M20" s="8"/>
       <c r="N20" s="12"/>
       <c r="O20" s="12">
@@ -1016,23 +1034,25 @@
         <v>12.0</v>
       </c>
       <c r="F21" s="8">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="H21" s="8" t="s">
         <v>45</v>
       </c>
       <c r="I21" s="12">
         <f>0.63*E16</f>
-        <v>37.8</v>
+        <v>88.2</v>
       </c>
       <c r="J21" s="4">
         <f>0.63*E26</f>
-        <v>15.12</v>
+        <v>30.24</v>
       </c>
       <c r="K21" s="12">
         <v>25.0</v>
       </c>
-      <c r="L21" s="12"/>
+      <c r="L21" s="12">
+        <v>28.0</v>
+      </c>
       <c r="M21" s="8"/>
       <c r="N21" s="12"/>
       <c r="O21" s="12">
@@ -1053,23 +1073,25 @@
         <v>12.0</v>
       </c>
       <c r="F22" s="8">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="H22" s="8" t="s">
         <v>47</v>
       </c>
       <c r="I22" s="12">
         <f>0.6*E16</f>
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="J22" s="4">
         <f>0.6*E26</f>
-        <v>14.4</v>
+        <v>28.8</v>
       </c>
       <c r="K22" s="12">
         <v>15.0</v>
       </c>
-      <c r="L22" s="12"/>
+      <c r="L22" s="12">
+        <v>18.0</v>
+      </c>
       <c r="M22" s="8"/>
       <c r="N22" s="12"/>
       <c r="O22" s="12">
@@ -1106,7 +1128,9 @@
       <c r="K23" s="12">
         <v>0.0</v>
       </c>
-      <c r="L23" s="12"/>
+      <c r="L23" s="12">
+        <v>0.0</v>
+      </c>
       <c r="M23" s="8"/>
       <c r="N23" s="12"/>
       <c r="O23" s="12">
@@ -1219,7 +1243,7 @@
       </c>
       <c r="E26" s="8">
         <f>12*MIN(SUM(F19:F25),COUNT(F19:F25)-2)</f>
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="F26" s="8"/>
       <c r="I26" s="7"/>

</xml_diff>

<commit_message>
posted 213 m3 gradelines
</commit_message>
<xml_diff>
--- a/213_S26/gradelines.xlsx
+++ b/213_S26/gradelines.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="52">
   <si>
     <t>Course</t>
   </si>
@@ -161,12 +161,6 @@
   </si>
   <si>
     <t>F</t>
-  </si>
-  <si>
-    <t>Q6</t>
-  </si>
-  <si>
-    <t>Q7</t>
   </si>
   <si>
     <t>Current Weight</t>
@@ -509,7 +503,7 @@
       </c>
       <c r="E2" s="4">
         <f>100*(SUM(F5:F15)/COUNT(F5:F15)*0.15 + SUM(F19:F25)/COUNT(F19:F25)*0.1 + SUM(F29:F31)*0.15 + F32*0.3)</f>
-        <v>45.25974026</v>
+        <v>68.63636364</v>
       </c>
     </row>
     <row r="3">
@@ -690,17 +684,17 @@
         <v>20.0</v>
       </c>
       <c r="F12" s="8">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>28</v>
       </c>
       <c r="I12" s="12">
         <f>0.93*E16</f>
-        <v>130.2</v>
+        <v>186</v>
       </c>
       <c r="J12" s="12">
-        <f>0.93*E26</f>
+        <f>0.93*E24</f>
         <v>44.64</v>
       </c>
       <c r="K12" s="12">
@@ -709,11 +703,13 @@
       <c r="L12" s="12">
         <v>70.0</v>
       </c>
-      <c r="M12" s="8"/>
+      <c r="M12" s="12">
+        <v>73.0</v>
+      </c>
       <c r="N12" s="12"/>
       <c r="O12" s="12">
-        <f>IF(E16=0, 0, I12/E16)*I25 + IF(E26=0, 0, J12/E26)*J25 + IF(E29=0, 0, K12/E29)*K25 + IF(E30=0, 0, L12/E30)*L25 + IF(E31=0, 0, M12/E31)*M25 + IF(E32=0, 0, N12/E32)*N25</f>
-        <v>89.99208145</v>
+        <f>IF(E16=0, 0, I12/E16)*I25 + IF(E24=0, 0, J12/E24)*J25 + IF(E29=0, 0, K12/E29)*K25 + IF(E30=0, 0, L12/E30)*L25 + IF(E31=0, 0, M12/E31)*M25 + IF(E32=0, 0, N12/E32)*N25</f>
+        <v>90.84598679</v>
       </c>
     </row>
     <row r="13">
@@ -729,17 +725,17 @@
         <v>20.0</v>
       </c>
       <c r="F13" s="8">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>30</v>
       </c>
       <c r="I13" s="12">
         <f>0.9*E16</f>
-        <v>126</v>
+        <v>180</v>
       </c>
       <c r="J13" s="4">
-        <f>0.9*E26</f>
+        <f>0.9*E24</f>
         <v>43.2</v>
       </c>
       <c r="K13" s="12">
@@ -748,11 +744,13 @@
       <c r="L13" s="12">
         <v>66.0</v>
       </c>
-      <c r="M13" s="8"/>
+      <c r="M13" s="12">
+        <v>68.0</v>
+      </c>
       <c r="N13" s="12"/>
       <c r="O13" s="12">
-        <f>IF(E16=0, 0, I13/E16)*I25 + IF(E26=0, 0, J13/E26)*J25 + IF(E29=0, 0, K13/E29)*K25 + IF(E30=0, 0, L13/E30)*L25 + IF(E31=0, 0, M13/E31)*M25 + IF(E32=0, 0, N13/E32)*N25</f>
-        <v>85.11312217</v>
+        <f>IF(E16=0, 0, I13/E16)*I25 + IF(E24=0, 0, J13/E24)*J25 + IF(E29=0, 0, K13/E29)*K25 + IF(E30=0, 0, L13/E30)*L25 + IF(E31=0, 0, M13/E31)*M25 + IF(E32=0, 0, N13/E32)*N25</f>
+        <v>85.76106879</v>
       </c>
     </row>
     <row r="14">
@@ -768,17 +766,17 @@
         <v>20.0</v>
       </c>
       <c r="F14" s="8">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="H14" s="8" t="s">
         <v>32</v>
       </c>
       <c r="I14" s="12">
         <f>0.87*E16</f>
-        <v>121.8</v>
+        <v>174</v>
       </c>
       <c r="J14" s="4">
-        <f>0.87*E26</f>
+        <f>0.87*E24</f>
         <v>41.76</v>
       </c>
       <c r="K14" s="12">
@@ -787,11 +785,13 @@
       <c r="L14" s="12">
         <v>62.0</v>
       </c>
-      <c r="M14" s="8"/>
+      <c r="M14" s="12">
+        <v>63.0</v>
+      </c>
       <c r="N14" s="12"/>
       <c r="O14" s="12">
-        <f>IF(E16=0, 0, I14/E16)*I25 + IF(E26=0, 0, J14/E26)*J25 + IF(E29=0, 0, K14/E29)*K25 + IF(E30=0, 0, L14/E30)*L25 + IF(E31=0, 0, M14/E31)*M25 + IF(E32=0, 0, N14/E32)*N25</f>
-        <v>80.2341629</v>
+        <f>IF(E16=0, 0, I14/E16)*I25 + IF(E24=0, 0, J14/E24)*J25 + IF(E29=0, 0, K14/E29)*K25 + IF(E30=0, 0, L14/E30)*L25 + IF(E31=0, 0, M14/E31)*M25 + IF(E32=0, 0, N14/E32)*N25</f>
+        <v>80.67615079</v>
       </c>
     </row>
     <row r="15">
@@ -814,10 +814,10 @@
       </c>
       <c r="I15" s="12">
         <f>0.83*E16</f>
-        <v>116.2</v>
+        <v>166</v>
       </c>
       <c r="J15" s="4">
-        <f>0.83*E26</f>
+        <f>0.83*E24</f>
         <v>39.84</v>
       </c>
       <c r="K15" s="12">
@@ -826,11 +826,13 @@
       <c r="L15" s="12">
         <v>58.0</v>
       </c>
-      <c r="M15" s="8"/>
+      <c r="M15" s="12">
+        <v>58.0</v>
+      </c>
       <c r="N15" s="12"/>
       <c r="O15" s="12">
-        <f>IF(E16=0, 0, I15/E16)*I25 + IF(E26=0, 0, J15/E26)*J25 + IF(E29=0, 0, K15/E29)*K25 + IF(E30=0, 0, L15/E30)*L25 + IF(E31=0, 0, M15/E31)*M25 + IF(E32=0, 0, N15/E32)*N25</f>
-        <v>75.10520362</v>
+        <f>IF(E16=0, 0, I15/E16)*I25 + IF(E24=0, 0, J15/E24)*J25 + IF(E29=0, 0, K15/E29)*K25 + IF(E30=0, 0, L15/E30)*L25 + IF(E31=0, 0, M15/E31)*M25 + IF(E32=0, 0, N15/E32)*N25</f>
+        <v>75.34123279</v>
       </c>
     </row>
     <row r="16">
@@ -846,7 +848,7 @@
       </c>
       <c r="E16" s="8">
         <f>20*MIN(SUM(F5:F15),COUNT(F5:F15)-1)</f>
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="F16" s="8"/>
       <c r="H16" s="8" t="s">
@@ -854,10 +856,10 @@
       </c>
       <c r="I16" s="12">
         <f>0.8*E16</f>
-        <v>112</v>
+        <v>160</v>
       </c>
       <c r="J16" s="4">
-        <f>0.8*E26</f>
+        <f>0.8*E24</f>
         <v>38.4</v>
       </c>
       <c r="K16" s="12">
@@ -866,11 +868,13 @@
       <c r="L16" s="12">
         <v>54.0</v>
       </c>
-      <c r="M16" s="8"/>
+      <c r="M16" s="12">
+        <v>53.0</v>
+      </c>
       <c r="N16" s="12"/>
       <c r="O16" s="12">
-        <f>IF(E16=0, 0, I16/E16)*I25 + IF(E26=0, 0, J16/E26)*J25 + IF(E29=0, 0, K16/E29)*K25 + IF(E30=0, 0, L16/E30)*L25 + IF(E31=0, 0, M16/E31)*M25 + IF(E32=0, 0, N16/E32)*N25</f>
-        <v>70.22624434</v>
+        <f>IF(E16=0, 0, I16/E16)*I25 + IF(E24=0, 0, J16/E24)*J25 + IF(E29=0, 0, K16/E29)*K25 + IF(E30=0, 0, L16/E30)*L25 + IF(E31=0, 0, M16/E31)*M25 + IF(E32=0, 0, N16/E32)*N25</f>
+        <v>70.25631479</v>
       </c>
     </row>
     <row r="17">
@@ -884,10 +888,10 @@
       </c>
       <c r="I17" s="4">
         <f>0.77*E16</f>
-        <v>107.8</v>
+        <v>154</v>
       </c>
       <c r="J17" s="4">
-        <f>0.77*E26</f>
+        <f>0.77*E24</f>
         <v>36.96</v>
       </c>
       <c r="K17" s="12">
@@ -896,11 +900,13 @@
       <c r="L17" s="12">
         <v>50.0</v>
       </c>
-      <c r="M17" s="8"/>
+      <c r="M17" s="12">
+        <v>47.0</v>
+      </c>
       <c r="N17" s="12"/>
       <c r="O17" s="12">
-        <f>IF(E16=0, 0, I17/E16)*I25 + IF(E26=0, 0, J17/E26)*J25 + IF(E29=0, 0, K17/E29)*K25 + IF(E30=0, 0, L17/E30)*L25 + IF(E31=0, 0, M17/E31)*M25 + IF(E32=0, 0, N17/E32)*N25</f>
-        <v>65.34728507</v>
+        <f>IF(E16=0, 0, I17/E16)*I25 + IF(E24=0, 0, J17/E24)*J25 + IF(E29=0, 0, K17/E29)*K25 + IF(E30=0, 0, L17/E30)*L25 + IF(E31=0, 0, M17/E31)*M25 + IF(E32=0, 0, N17/E32)*N25</f>
+        <v>64.8549411</v>
       </c>
     </row>
     <row r="18">
@@ -924,10 +930,10 @@
       </c>
       <c r="I18" s="4">
         <f>0.73*E16</f>
-        <v>102.2</v>
+        <v>146</v>
       </c>
       <c r="J18" s="4">
-        <f>0.73*E26</f>
+        <f>0.73*E24</f>
         <v>35.04</v>
       </c>
       <c r="K18" s="12">
@@ -936,11 +942,13 @@
       <c r="L18" s="12">
         <v>46.0</v>
       </c>
-      <c r="M18" s="8"/>
+      <c r="M18" s="12">
+        <v>41.0</v>
+      </c>
       <c r="N18" s="12"/>
       <c r="O18" s="12">
-        <f>IF(E16=0, 0, I18/E16)*I25 + IF(E26=0, 0, J18/E26)*J25 + IF(E29=0, 0, K18/E29)*K25 + IF(E30=0, 0, L18/E30)*L25 + IF(E31=0, 0, M18/E31)*M25 + IF(E32=0, 0, N18/E32)*N25</f>
-        <v>59.77714932</v>
+        <f>IF(E16=0, 0, I18/E16)*I25 + IF(E24=0, 0, J18/E24)*J25 + IF(E29=0, 0, K18/E29)*K25 + IF(E30=0, 0, L18/E30)*L25 + IF(E31=0, 0, M18/E31)*M25 + IF(E32=0, 0, N18/E32)*N25</f>
+        <v>58.90944976</v>
       </c>
     </row>
     <row r="19">
@@ -949,7 +957,7 @@
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="8">
-        <f t="shared" ref="D19:D25" si="2">C19/E19*12</f>
+        <f t="shared" ref="D19:D23" si="2">C19/E19*12</f>
         <v>0</v>
       </c>
       <c r="E19" s="8">
@@ -963,10 +971,10 @@
       </c>
       <c r="I19" s="12">
         <f>0.7*E16</f>
-        <v>98</v>
+        <v>140</v>
       </c>
       <c r="J19" s="4">
-        <f>0.7*E26</f>
+        <f>0.7*E24</f>
         <v>33.6</v>
       </c>
       <c r="K19" s="12">
@@ -975,11 +983,13 @@
       <c r="L19" s="12">
         <v>40.0</v>
       </c>
-      <c r="M19" s="8"/>
+      <c r="M19" s="12">
+        <v>35.0</v>
+      </c>
       <c r="N19" s="12"/>
       <c r="O19" s="12">
-        <f>IF(E16=0, 0, I19/E16)*I25 + IF(E26=0, 0, J19/E26)*J25 + IF(E29=0, 0, K19/E29)*K25 + IF(E30=0, 0, L19/E30)*L25 + IF(E31=0, 0, M19/E31)*M25 + IF(E32=0, 0, N19/E32)*N25</f>
-        <v>53.49547511</v>
+        <f>IF(E16=0, 0, I19/E16)*I25 + IF(E24=0, 0, J19/E24)*J25 + IF(E29=0, 0, K19/E29)*K25 + IF(E30=0, 0, L19/E30)*L25 + IF(E31=0, 0, M19/E31)*M25 + IF(E32=0, 0, N19/E32)*N25</f>
+        <v>52.57293278</v>
       </c>
     </row>
     <row r="20">
@@ -1002,10 +1012,10 @@
       </c>
       <c r="I20" s="12">
         <f>0.67*E16</f>
-        <v>93.8</v>
+        <v>134</v>
       </c>
       <c r="J20" s="4">
-        <f>0.67*E26</f>
+        <f>0.67*E24</f>
         <v>32.16</v>
       </c>
       <c r="K20" s="12">
@@ -1014,11 +1024,13 @@
       <c r="L20" s="12">
         <v>34.0</v>
       </c>
-      <c r="M20" s="8"/>
+      <c r="M20" s="12">
+        <v>28.0</v>
+      </c>
       <c r="N20" s="12"/>
       <c r="O20" s="12">
-        <f>IF(E16=0, 0, I20/E16)*I25 + IF(E26=0, 0, J20/E26)*J25 + IF(E29=0, 0, K20/E29)*K25 + IF(E30=0, 0, L20/E30)*L25 + IF(E31=0, 0, M20/E31)*M25 + IF(E32=0, 0, N20/E32)*N25</f>
-        <v>47.2138009</v>
+        <f>IF(E16=0, 0, I20/E16)*I25 + IF(E24=0, 0, J20/E24)*J25 + IF(E29=0, 0, K20/E29)*K25 + IF(E30=0, 0, L20/E30)*L25 + IF(E31=0, 0, M20/E31)*M25 + IF(E32=0, 0, N20/E32)*N25</f>
+        <v>45.9199601</v>
       </c>
     </row>
     <row r="21">
@@ -1041,10 +1053,10 @@
       </c>
       <c r="I21" s="12">
         <f>0.63*E16</f>
-        <v>88.2</v>
+        <v>126</v>
       </c>
       <c r="J21" s="4">
-        <f>0.63*E26</f>
+        <f>0.63*E24</f>
         <v>30.24</v>
       </c>
       <c r="K21" s="12">
@@ -1053,11 +1065,13 @@
       <c r="L21" s="12">
         <v>28.0</v>
       </c>
-      <c r="M21" s="8"/>
+      <c r="M21" s="12">
+        <v>20.0</v>
+      </c>
       <c r="N21" s="12"/>
       <c r="O21" s="12">
-        <f>IF(E16=0, 0, I21/E16)*I25 + IF(E26=0, 0, J21/E26)*J25 + IF(E29=0, 0, K21/E29)*K25 + IF(E30=0, 0, L21/E30)*L25 + IF(E31=0, 0, M21/E31)*M25 + IF(E32=0, 0, N21/E32)*N25</f>
-        <v>40.24095023</v>
+        <f>IF(E16=0, 0, I21/E16)*I25 + IF(E24=0, 0, J21/E24)*J25 + IF(E29=0, 0, K21/E29)*K25 + IF(E30=0, 0, L21/E30)*L25 + IF(E31=0, 0, M21/E31)*M25 + IF(E32=0, 0, N21/E32)*N25</f>
+        <v>38.40641407</v>
       </c>
     </row>
     <row r="22">
@@ -1080,10 +1094,10 @@
       </c>
       <c r="I22" s="12">
         <f>0.6*E16</f>
-        <v>84</v>
+        <v>120</v>
       </c>
       <c r="J22" s="4">
-        <f>0.6*E26</f>
+        <f>0.6*E24</f>
         <v>28.8</v>
       </c>
       <c r="K22" s="12">
@@ -1092,11 +1106,13 @@
       <c r="L22" s="12">
         <v>18.0</v>
       </c>
-      <c r="M22" s="8"/>
+      <c r="M22" s="12">
+        <v>10.0</v>
+      </c>
       <c r="N22" s="12"/>
       <c r="O22" s="12">
-        <f>IF(E16=0, 0, I22/E16)*I25 + IF(E26=0, 0, J22/E26)*J25 + IF(E29=0, 0, K22/E29)*K25 + IF(E30=0, 0, L22/E30)*L25 + IF(E31=0, 0, M22/E31)*M25 + IF(E32=0, 0, N22/E32)*N25</f>
-        <v>30.27149321</v>
+        <f>IF(E16=0, 0, I22/E16)*I25 + IF(E24=0, 0, J22/E24)*J25 + IF(E29=0, 0, K22/E29)*K25 + IF(E30=0, 0, L22/E30)*L25 + IF(E31=0, 0, M22/E31)*M25 + IF(E32=0, 0, N22/E32)*N25</f>
+        <v>28.34555244</v>
       </c>
     </row>
     <row r="23">
@@ -1112,7 +1128,7 @@
         <v>12.0</v>
       </c>
       <c r="F23" s="8">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="H23" s="8" t="s">
         <v>49</v>
@@ -1122,7 +1138,7 @@
         <v>0</v>
       </c>
       <c r="J23" s="4">
-        <f>0*E26</f>
+        <f>0*E24</f>
         <v>0</v>
       </c>
       <c r="K23" s="12">
@@ -1131,28 +1147,31 @@
       <c r="L23" s="12">
         <v>0.0</v>
       </c>
-      <c r="M23" s="8"/>
+      <c r="M23" s="12">
+        <v>0.0</v>
+      </c>
       <c r="N23" s="12"/>
       <c r="O23" s="12">
-        <f>IF(E16=0, 0, I23/E16)*I25 + IF(E26=0, 0, J23/E26)*J25 + IF(E29=0, 0, K23/E29)*K25 + IF(E30=0, 0, L23/E30)*L25 + IF(E31=0, 0, M23/E31)*M25 + IF(E32=0, 0, N23/E32)*N25</f>
+        <f>IF(E16=0, 0, I23/E16)*I25 + IF(E24=0, 0, J23/E24)*J25 + IF(E29=0, 0, K23/E29)*K25 + IF(E30=0, 0, L23/E30)*L25 + IF(E31=0, 0, M23/E31)*M25 + IF(E32=0, 0, N23/E32)*N25</f>
         <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C24" s="9"/>
+        <v>35</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>36</v>
+      </c>
       <c r="D24" s="8">
-        <f t="shared" si="2"/>
+        <f t="array" ref="D24">SUM(IFERROR(LARGE(D19:D23,{1,2,3,4}),0))</f>
         <v>0</v>
       </c>
       <c r="E24" s="8">
-        <v>12.0</v>
-      </c>
-      <c r="F24" s="8">
-        <v>0.0</v>
-      </c>
+        <f>12*MIN(SUM(F19:F25),COUNT(F19:F23)-1)</f>
+        <v>48</v>
+      </c>
+      <c r="F24" s="8"/>
       <c r="H24" s="8" t="s">
         <v>7</v>
       </c>
@@ -1161,7 +1180,7 @@
         <v>0</v>
       </c>
       <c r="J24" s="12">
-        <f>D26</f>
+        <f>D24</f>
         <v>0</v>
       </c>
       <c r="K24" s="12" t="str">
@@ -1181,27 +1200,18 @@
         <v/>
       </c>
       <c r="O24" s="12">
-        <f>IF(E16=0, 0, I24/E16)*I25 + IF(E26=0, 0, J24/E26)*J25 + IF(E29=0, 0, K24/E29)*K25 + IF(E30=0, 0, L24/E30)*L25 + IF(E31=0, 0, M24/E31)*M25 + IF(E32=0, 0, N24/E32)*N25</f>
+        <f>IF(E16=0, 0, I24/E16)*I25 + IF(E24=0, 0, J24/E24)*J25 + IF(E29=0, 0, K24/E29)*K25 + IF(E30=0, 0, L24/E30)*L25 + IF(E31=0, 0, M24/E31)*M25 + IF(E32=0, 0, N24/E32)*N25</f>
         <v>0</v>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="8">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E25" s="8">
-        <v>12.0</v>
-      </c>
-      <c r="F25" s="8">
-        <v>0.0</v>
-      </c>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
       <c r="H25" s="8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I25" s="12">
         <v>15.0</v>
@@ -1211,15 +1221,15 @@
       </c>
       <c r="K25" s="12">
         <f>75*F29/(F29+F30+F31+2*F32)</f>
-        <v>37.5</v>
+        <v>25</v>
       </c>
       <c r="L25" s="12">
         <f>75*F30/(F29+F30+F31+2*F32)</f>
-        <v>37.5</v>
+        <v>25</v>
       </c>
       <c r="M25" s="12">
         <f>75*F31/(F29+F30+F31+2*F32)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="N25" s="12">
         <f>75*2*F32/(F29+F30+F31+2*F32)</f>
@@ -1231,21 +1241,6 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" s="8">
-        <f t="array" ref="D26">SUM(IFERROR(LARGE(D19:D25,{1,2,3,4,5,6,7}),0))</f>
-        <v>0</v>
-      </c>
-      <c r="E26" s="8">
-        <f>12*MIN(SUM(F19:F25),COUNT(F19:F25)-2)</f>
-        <v>48</v>
-      </c>
-      <c r="F26" s="8"/>
       <c r="I26" s="7"/>
       <c r="J26" s="7"/>
       <c r="K26" s="7"/>
@@ -1259,7 +1254,7 @@
     </row>
     <row r="28">
       <c r="B28" s="11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>7</v>
@@ -1317,10 +1312,10 @@
         <v>36</v>
       </c>
       <c r="E31" s="8">
-        <v>0.0</v>
+        <v>79.0</v>
       </c>
       <c r="F31" s="8">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="32">

</xml_diff>

<commit_message>
updated Math 213 gradelines
</commit_message>
<xml_diff>
--- a/213_S26/gradelines.xlsx
+++ b/213_S26/gradelines.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Gradelines Including Final Exam" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Pre-Final Exam Gradelines" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="52">
   <si>
     <t>Course</t>
   </si>
@@ -176,7 +177,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.##"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -201,6 +202,21 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -222,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -258,6 +274,39 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -267,6 +316,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -503,7 +556,7 @@
       </c>
       <c r="E2" s="4">
         <f>100*(SUM(F5:F15)/COUNT(F5:F15)*0.15 + SUM(F19:F25)/COUNT(F19:F25)*0.1 + SUM(F29:F31)*0.15 + F32*0.3)</f>
-        <v>68.63636364</v>
+        <v>98.63636364</v>
       </c>
     </row>
     <row r="3">
@@ -706,10 +759,12 @@
       <c r="M12" s="12">
         <v>73.0</v>
       </c>
-      <c r="N12" s="12"/>
+      <c r="N12" s="13">
+        <v>111.0</v>
+      </c>
       <c r="O12" s="12">
         <f>IF(E16=0, 0, I12/E16)*I25 + IF(E24=0, 0, J12/E24)*J25 + IF(E29=0, 0, K12/E29)*K25 + IF(E30=0, 0, L12/E30)*L25 + IF(E31=0, 0, M12/E31)*M25 + IF(E32=0, 0, N12/E32)*N25</f>
-        <v>90.84598679</v>
+        <v>90.8807628</v>
       </c>
     </row>
     <row r="13">
@@ -747,10 +802,12 @@
       <c r="M13" s="12">
         <v>68.0</v>
       </c>
-      <c r="N13" s="12"/>
+      <c r="N13" s="13">
+        <v>104.0</v>
+      </c>
       <c r="O13" s="12">
         <f>IF(E16=0, 0, I13/E16)*I25 + IF(E24=0, 0, J13/E24)*J25 + IF(E29=0, 0, K13/E29)*K25 + IF(E30=0, 0, L13/E30)*L25 + IF(E31=0, 0, M13/E31)*M25 + IF(E32=0, 0, N13/E32)*N25</f>
-        <v>85.76106879</v>
+        <v>85.82249493</v>
       </c>
     </row>
     <row r="14">
@@ -788,10 +845,12 @@
       <c r="M14" s="12">
         <v>63.0</v>
       </c>
-      <c r="N14" s="12"/>
+      <c r="N14" s="13">
+        <v>97.0</v>
+      </c>
       <c r="O14" s="12">
         <f>IF(E16=0, 0, I14/E16)*I25 + IF(E24=0, 0, J14/E24)*J25 + IF(E29=0, 0, K14/E29)*K25 + IF(E30=0, 0, L14/E30)*L25 + IF(E31=0, 0, M14/E31)*M25 + IF(E32=0, 0, N14/E32)*N25</f>
-        <v>80.67615079</v>
+        <v>80.76422706</v>
       </c>
     </row>
     <row r="15">
@@ -829,10 +888,12 @@
       <c r="M15" s="12">
         <v>58.0</v>
       </c>
-      <c r="N15" s="12"/>
+      <c r="N15" s="13">
+        <v>89.0</v>
+      </c>
       <c r="O15" s="12">
         <f>IF(E16=0, 0, I15/E16)*I25 + IF(E24=0, 0, J15/E24)*J25 + IF(E29=0, 0, K15/E29)*K25 + IF(E30=0, 0, L15/E30)*L25 + IF(E31=0, 0, M15/E31)*M25 + IF(E32=0, 0, N15/E32)*N25</f>
-        <v>75.34123279</v>
+        <v>75.21205675</v>
       </c>
     </row>
     <row r="16">
@@ -871,10 +932,12 @@
       <c r="M16" s="12">
         <v>53.0</v>
       </c>
-      <c r="N16" s="12"/>
+      <c r="N16" s="13">
+        <v>81.0</v>
+      </c>
       <c r="O16" s="12">
         <f>IF(E16=0, 0, I16/E16)*I25 + IF(E24=0, 0, J16/E24)*J25 + IF(E29=0, 0, K16/E29)*K25 + IF(E30=0, 0, L16/E30)*L25 + IF(E31=0, 0, M16/E31)*M25 + IF(E32=0, 0, N16/E32)*N25</f>
-        <v>70.25631479</v>
+        <v>69.90988644</v>
       </c>
     </row>
     <row r="17">
@@ -903,10 +966,12 @@
       <c r="M17" s="12">
         <v>47.0</v>
       </c>
-      <c r="N17" s="12"/>
+      <c r="N17" s="13">
+        <v>73.0</v>
+      </c>
       <c r="O17" s="12">
         <f>IF(E16=0, 0, I17/E16)*I25 + IF(E24=0, 0, J17/E24)*J25 + IF(E29=0, 0, K17/E29)*K25 + IF(E30=0, 0, L17/E30)*L25 + IF(E31=0, 0, M17/E31)*M25 + IF(E32=0, 0, N17/E32)*N25</f>
-        <v>64.8549411</v>
+        <v>64.41784271</v>
       </c>
     </row>
     <row r="18">
@@ -945,10 +1010,12 @@
       <c r="M18" s="12">
         <v>41.0</v>
       </c>
-      <c r="N18" s="12"/>
+      <c r="N18" s="13">
+        <v>65.0</v>
+      </c>
       <c r="O18" s="12">
         <f>IF(E16=0, 0, I18/E16)*I25 + IF(E24=0, 0, J18/E24)*J25 + IF(E29=0, 0, K18/E29)*K25 + IF(E30=0, 0, L18/E30)*L25 + IF(E31=0, 0, M18/E31)*M25 + IF(E32=0, 0, N18/E32)*N25</f>
-        <v>58.90944976</v>
+        <v>58.49932839</v>
       </c>
     </row>
     <row r="19">
@@ -986,10 +1053,12 @@
       <c r="M19" s="12">
         <v>35.0</v>
       </c>
-      <c r="N19" s="12"/>
+      <c r="N19" s="13">
+        <v>57.0</v>
+      </c>
       <c r="O19" s="12">
         <f>IF(E16=0, 0, I19/E16)*I25 + IF(E24=0, 0, J19/E24)*J25 + IF(E29=0, 0, K19/E29)*K25 + IF(E30=0, 0, L19/E30)*L25 + IF(E31=0, 0, M19/E31)*M25 + IF(E32=0, 0, N19/E32)*N25</f>
-        <v>52.57293278</v>
+        <v>52.44619869</v>
       </c>
     </row>
     <row r="20">
@@ -1027,10 +1096,12 @@
       <c r="M20" s="12">
         <v>28.0</v>
       </c>
-      <c r="N20" s="12"/>
+      <c r="N20" s="13">
+        <v>47.0</v>
+      </c>
       <c r="O20" s="12">
         <f>IF(E16=0, 0, I20/E16)*I25 + IF(E24=0, 0, J20/E24)*J25 + IF(E29=0, 0, K20/E29)*K25 + IF(E30=0, 0, L20/E30)*L25 + IF(E31=0, 0, M20/E31)*M25 + IF(E32=0, 0, N20/E32)*N25</f>
-        <v>45.9199601</v>
+        <v>45.71539069</v>
       </c>
     </row>
     <row r="21">
@@ -1068,10 +1139,12 @@
       <c r="M21" s="12">
         <v>20.0</v>
       </c>
-      <c r="N21" s="12"/>
+      <c r="N21" s="13">
+        <v>35.0</v>
+      </c>
       <c r="O21" s="12">
         <f>IF(E16=0, 0, I21/E16)*I25 + IF(E24=0, 0, J21/E24)*J25 + IF(E29=0, 0, K21/E29)*K25 + IF(E30=0, 0, L21/E30)*L25 + IF(E31=0, 0, M21/E31)*M25 + IF(E32=0, 0, N21/E32)*N25</f>
-        <v>38.40641407</v>
+        <v>37.88043381</v>
       </c>
     </row>
     <row r="22">
@@ -1109,10 +1182,12 @@
       <c r="M22" s="12">
         <v>10.0</v>
       </c>
-      <c r="N22" s="12"/>
+      <c r="N22" s="13">
+        <v>20.0</v>
+      </c>
       <c r="O22" s="12">
         <f>IF(E16=0, 0, I22/E16)*I25 + IF(E24=0, 0, J22/E24)*J25 + IF(E29=0, 0, K22/E29)*K25 + IF(E30=0, 0, L22/E30)*L25 + IF(E31=0, 0, M22/E31)*M25 + IF(E32=0, 0, N22/E32)*N25</f>
-        <v>28.34555244</v>
+        <v>27.88538024</v>
       </c>
     </row>
     <row r="23">
@@ -1150,7 +1225,9 @@
       <c r="M23" s="12">
         <v>0.0</v>
       </c>
-      <c r="N23" s="12"/>
+      <c r="N23" s="13">
+        <v>0.0</v>
+      </c>
       <c r="O23" s="12">
         <f>IF(E16=0, 0, I23/E16)*I25 + IF(E24=0, 0, J23/E24)*J25 + IF(E29=0, 0, K23/E29)*K25 + IF(E30=0, 0, L23/E30)*L25 + IF(E31=0, 0, M23/E31)*M25 + IF(E32=0, 0, N23/E32)*N25</f>
         <v>0</v>
@@ -1221,19 +1298,19 @@
       </c>
       <c r="K25" s="12">
         <f>75*F29/(F29+F30+F31+2*F32)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="L25" s="12">
         <f>75*F30/(F29+F30+F31+2*F32)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="M25" s="12">
         <f>75*F31/(F29+F30+F31+2*F32)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="N25" s="12">
         <f>75*2*F32/(F29+F30+F31+2*F32)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="O25" s="12">
         <f>SUM(I25:N25)</f>
@@ -1327,14 +1404,1436 @@
         <v>36</v>
       </c>
       <c r="E32" s="8">
-        <v>0.0</v>
+        <v>123.0</v>
       </c>
       <c r="F32" s="8">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="33">
       <c r="D33" s="8"/>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="6" width="9.75"/>
+    <col customWidth="1" min="7" max="7" width="5.63"/>
+    <col customWidth="1" min="8" max="13" width="10.5"/>
+    <col customWidth="1" min="14" max="14" width="13.75"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="16"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
+      <c r="Q1" s="15"/>
+      <c r="R1" s="15"/>
+      <c r="S1" s="15"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="16"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="13">
+        <f>100*(SUM(F5:F15)/COUNT(F5:F15)*0.15 + SUM(F19:F25)/COUNT(F19:F25)*0.1 + SUM(F29:F31)*0.15 + F32*0.3)</f>
+        <v>70</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15"/>
+      <c r="N2" s="15"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="15"/>
+      <c r="S2" s="15"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="15"/>
+      <c r="Q3" s="15"/>
+      <c r="R3" s="15"/>
+      <c r="S3" s="15"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="15"/>
+      <c r="B4" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
+      <c r="R4" s="15"/>
+      <c r="S4" s="15"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="15"/>
+      <c r="B5" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="20"/>
+      <c r="D5" s="19">
+        <f t="shared" ref="D5:D15" si="1">C5/E5*20</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="F5" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+      <c r="R5" s="15"/>
+      <c r="S5" s="15"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="15"/>
+      <c r="B6" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="20"/>
+      <c r="D6" s="19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="F6" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="15"/>
+      <c r="R6" s="15"/>
+      <c r="S6" s="15"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="15"/>
+      <c r="B7" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="20"/>
+      <c r="D7" s="19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E7" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="F7" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G7" s="15"/>
+      <c r="H7" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="15"/>
+      <c r="N7" s="15"/>
+      <c r="O7" s="15"/>
+      <c r="P7" s="15"/>
+      <c r="Q7" s="15"/>
+      <c r="R7" s="15"/>
+      <c r="S7" s="15"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="15"/>
+      <c r="B8" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="20"/>
+      <c r="D8" s="19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E8" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="F8" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+      <c r="O8" s="15"/>
+      <c r="P8" s="15"/>
+      <c r="Q8" s="15"/>
+      <c r="R8" s="15"/>
+      <c r="S8" s="15"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="15"/>
+      <c r="B9" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="20"/>
+      <c r="D9" s="19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E9" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="F9" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
+      <c r="M9" s="15"/>
+      <c r="N9" s="15"/>
+      <c r="O9" s="15"/>
+      <c r="P9" s="15"/>
+      <c r="Q9" s="15"/>
+      <c r="R9" s="15"/>
+      <c r="S9" s="15"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="15"/>
+      <c r="B10" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="20"/>
+      <c r="D10" s="19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E10" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="F10" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="15"/>
+      <c r="O10" s="15"/>
+      <c r="P10" s="15"/>
+      <c r="Q10" s="15"/>
+      <c r="R10" s="15"/>
+      <c r="S10" s="15"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="15"/>
+      <c r="B11" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="20"/>
+      <c r="D11" s="19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E11" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="F11" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G11" s="15"/>
+      <c r="H11" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="J11" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="K11" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="L11" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="M11" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="N11" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="O11" s="16"/>
+      <c r="P11" s="15"/>
+      <c r="Q11" s="15"/>
+      <c r="R11" s="15"/>
+      <c r="S11" s="15"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="15"/>
+      <c r="B12" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="20"/>
+      <c r="D12" s="19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E12" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="F12" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G12" s="15"/>
+      <c r="H12" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I12" s="13">
+        <f>0.93*E16</f>
+        <v>186</v>
+      </c>
+      <c r="J12" s="13">
+        <f>0.93*E24</f>
+        <v>44.64</v>
+      </c>
+      <c r="K12" s="13">
+        <v>75.0</v>
+      </c>
+      <c r="L12" s="13">
+        <v>70.0</v>
+      </c>
+      <c r="M12" s="13">
+        <v>73.0</v>
+      </c>
+      <c r="N12" s="13">
+        <f>IF(E16=0, 0, I12/E16)*I25 + IF(E24=0, 0, J12/E24)*J25 + IF(E29=0, 0, K12/E29)*K25 + IF(E30=0, 0, L12/E30)*L25 + IF(E31=0, 0, M12/E31)*M25</f>
+        <v>90.84598679</v>
+      </c>
+      <c r="O12" s="15"/>
+      <c r="P12" s="15"/>
+      <c r="Q12" s="15"/>
+      <c r="R12" s="15"/>
+      <c r="S12" s="15"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="15"/>
+      <c r="B13" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="20"/>
+      <c r="D13" s="19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E13" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="F13" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G13" s="15"/>
+      <c r="H13" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="I13" s="13">
+        <f>0.9*E16</f>
+        <v>180</v>
+      </c>
+      <c r="J13" s="13">
+        <f>0.9*E24</f>
+        <v>43.2</v>
+      </c>
+      <c r="K13" s="13">
+        <v>70.0</v>
+      </c>
+      <c r="L13" s="13">
+        <v>66.0</v>
+      </c>
+      <c r="M13" s="13">
+        <v>68.0</v>
+      </c>
+      <c r="N13" s="13">
+        <f>IF(E16=0, 0, I13/E16)*I25 + IF(E24=0, 0, J13/E24)*J25 + IF(E29=0, 0, K13/E29)*K25 + IF(E30=0, 0, L13/E30)*L25 + IF(E31=0, 0, M13/E31)*M25</f>
+        <v>85.76106879</v>
+      </c>
+      <c r="O13" s="16"/>
+      <c r="P13" s="15"/>
+      <c r="Q13" s="15"/>
+      <c r="R13" s="15"/>
+      <c r="S13" s="15"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="15"/>
+      <c r="B14" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="20"/>
+      <c r="D14" s="19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E14" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="F14" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G14" s="15"/>
+      <c r="H14" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="I14" s="13">
+        <f>0.87*E16</f>
+        <v>174</v>
+      </c>
+      <c r="J14" s="13">
+        <f>0.87*E24</f>
+        <v>41.76</v>
+      </c>
+      <c r="K14" s="13">
+        <v>65.0</v>
+      </c>
+      <c r="L14" s="13">
+        <v>62.0</v>
+      </c>
+      <c r="M14" s="13">
+        <v>63.0</v>
+      </c>
+      <c r="N14" s="13">
+        <f>IF(E16=0, 0, I14/E16)*I25 + IF(E24=0, 0, J14/E24)*J25 + IF(E29=0, 0, K14/E29)*K25 + IF(E30=0, 0, L14/E30)*L25 + IF(E31=0, 0, M14/E31)*M25</f>
+        <v>80.67615079</v>
+      </c>
+      <c r="O14" s="15"/>
+      <c r="P14" s="15"/>
+      <c r="Q14" s="15"/>
+      <c r="R14" s="15"/>
+      <c r="S14" s="15"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="15"/>
+      <c r="B15" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="20"/>
+      <c r="D15" s="19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E15" s="19">
+        <v>20.0</v>
+      </c>
+      <c r="F15" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="G15" s="15"/>
+      <c r="H15" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I15" s="13">
+        <f>0.83*E16</f>
+        <v>166</v>
+      </c>
+      <c r="J15" s="13">
+        <f>0.83*E24</f>
+        <v>39.84</v>
+      </c>
+      <c r="K15" s="13">
+        <v>60.0</v>
+      </c>
+      <c r="L15" s="13">
+        <v>58.0</v>
+      </c>
+      <c r="M15" s="13">
+        <v>58.0</v>
+      </c>
+      <c r="N15" s="13">
+        <f>IF(E16=0, 0, I15/E16)*I25 + IF(E24=0, 0, J15/E24)*J25 + IF(E29=0, 0, K15/E29)*K25 + IF(E30=0, 0, L15/E30)*L25 + IF(E31=0, 0, M15/E31)*M25</f>
+        <v>75.34123279</v>
+      </c>
+      <c r="O15" s="15"/>
+      <c r="P15" s="15"/>
+      <c r="Q15" s="15"/>
+      <c r="R15" s="15"/>
+      <c r="S15" s="15"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="15"/>
+      <c r="B16" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="19">
+        <f t="array" ref="D16">SUM(IFERROR(LARGE(D5:D15,{1,2,3,4,5,6,7,8,9,10}),0))</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="19">
+        <f>20*MIN(SUM(F5:F15),COUNT(F5:F15)-1)</f>
+        <v>200</v>
+      </c>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="I16" s="13">
+        <f>0.8*E16</f>
+        <v>160</v>
+      </c>
+      <c r="J16" s="13">
+        <f>0.8*E24</f>
+        <v>38.4</v>
+      </c>
+      <c r="K16" s="13">
+        <v>55.0</v>
+      </c>
+      <c r="L16" s="13">
+        <v>54.0</v>
+      </c>
+      <c r="M16" s="13">
+        <v>53.0</v>
+      </c>
+      <c r="N16" s="13">
+        <f>IF(E16=0, 0, I16/E16)*I25 + IF(E24=0, 0, J16/E24)*J25 + IF(E29=0, 0, K16/E29)*K25 + IF(E30=0, 0, L16/E30)*L25 + IF(E31=0, 0, M16/E31)*M25</f>
+        <v>70.25631479</v>
+      </c>
+      <c r="O16" s="15"/>
+      <c r="P16" s="15"/>
+      <c r="Q16" s="15"/>
+      <c r="R16" s="15"/>
+      <c r="S16" s="15"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="I17" s="13">
+        <f>0.77*E16</f>
+        <v>154</v>
+      </c>
+      <c r="J17" s="13">
+        <f>0.77*E24</f>
+        <v>36.96</v>
+      </c>
+      <c r="K17" s="13">
+        <v>50.0</v>
+      </c>
+      <c r="L17" s="13">
+        <v>50.0</v>
+      </c>
+      <c r="M17" s="13">
+        <v>47.0</v>
+      </c>
+      <c r="N17" s="13">
+        <f>IF(E16=0, 0, I17/E16)*I25 + IF(E24=0, 0, J17/E24)*J25 + IF(E29=0, 0, K17/E29)*K25 + IF(E30=0, 0, L17/E30)*L25 + IF(E31=0, 0, M17/E31)*M25</f>
+        <v>64.8549411</v>
+      </c>
+      <c r="O17" s="15"/>
+      <c r="P17" s="15"/>
+      <c r="Q17" s="15"/>
+      <c r="R17" s="15"/>
+      <c r="S17" s="15"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="15"/>
+      <c r="B18" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="15"/>
+      <c r="H18" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="I18" s="13">
+        <f>0.73*E16</f>
+        <v>146</v>
+      </c>
+      <c r="J18" s="13">
+        <f>0.73*E24</f>
+        <v>35.04</v>
+      </c>
+      <c r="K18" s="13">
+        <v>44.0</v>
+      </c>
+      <c r="L18" s="13">
+        <v>46.0</v>
+      </c>
+      <c r="M18" s="13">
+        <v>41.0</v>
+      </c>
+      <c r="N18" s="13">
+        <f>IF(E16=0, 0, I18/E16)*I25 + IF(E24=0, 0, J18/E24)*J25 + IF(E29=0, 0, K18/E29)*K25 + IF(E30=0, 0, L18/E30)*L25 + IF(E31=0, 0, M18/E31)*M25</f>
+        <v>58.90944976</v>
+      </c>
+      <c r="O18" s="15"/>
+      <c r="P18" s="15"/>
+      <c r="Q18" s="15"/>
+      <c r="R18" s="15"/>
+      <c r="S18" s="15"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="15"/>
+      <c r="B19" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="20"/>
+      <c r="D19" s="19">
+        <f t="shared" ref="D19:D23" si="2">C19/E19*12</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="19">
+        <v>12.0</v>
+      </c>
+      <c r="F19" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G19" s="15"/>
+      <c r="H19" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="I19" s="13">
+        <f>0.7*E16</f>
+        <v>140</v>
+      </c>
+      <c r="J19" s="13">
+        <f>0.7*E24</f>
+        <v>33.6</v>
+      </c>
+      <c r="K19" s="13">
+        <v>38.0</v>
+      </c>
+      <c r="L19" s="13">
+        <v>40.0</v>
+      </c>
+      <c r="M19" s="13">
+        <v>35.0</v>
+      </c>
+      <c r="N19" s="13">
+        <f>IF(E16=0, 0, I19/E16)*I25 + IF(E24=0, 0, J19/E24)*J25 + IF(E29=0, 0, K19/E29)*K25 + IF(E30=0, 0, L19/E30)*L25 + IF(E31=0, 0, M19/E31)*M25</f>
+        <v>52.57293278</v>
+      </c>
+      <c r="O19" s="15"/>
+      <c r="P19" s="15"/>
+      <c r="Q19" s="15"/>
+      <c r="R19" s="15"/>
+      <c r="S19" s="15"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15"/>
+      <c r="B20" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="20"/>
+      <c r="D20" s="19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E20" s="19">
+        <v>12.0</v>
+      </c>
+      <c r="F20" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G20" s="15"/>
+      <c r="H20" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="I20" s="13">
+        <f>0.67*E16</f>
+        <v>134</v>
+      </c>
+      <c r="J20" s="13">
+        <f>0.67*E24</f>
+        <v>32.16</v>
+      </c>
+      <c r="K20" s="13">
+        <v>32.0</v>
+      </c>
+      <c r="L20" s="13">
+        <v>34.0</v>
+      </c>
+      <c r="M20" s="13">
+        <v>28.0</v>
+      </c>
+      <c r="N20" s="13">
+        <f>IF(E16=0, 0, I20/E16)*I25 + IF(E24=0, 0, J20/E24)*J25 + IF(E29=0, 0, K20/E29)*K25 + IF(E30=0, 0, L20/E30)*L25 + IF(E31=0, 0, M20/E31)*M25</f>
+        <v>45.9199601</v>
+      </c>
+      <c r="O20" s="15"/>
+      <c r="P20" s="15"/>
+      <c r="Q20" s="15"/>
+      <c r="R20" s="15"/>
+      <c r="S20" s="15"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="15"/>
+      <c r="B21" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="20"/>
+      <c r="D21" s="19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E21" s="19">
+        <v>12.0</v>
+      </c>
+      <c r="F21" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G21" s="15"/>
+      <c r="H21" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="I21" s="13">
+        <f>0.63*E16</f>
+        <v>126</v>
+      </c>
+      <c r="J21" s="13">
+        <f>0.63*E24</f>
+        <v>30.24</v>
+      </c>
+      <c r="K21" s="13">
+        <v>25.0</v>
+      </c>
+      <c r="L21" s="13">
+        <v>28.0</v>
+      </c>
+      <c r="M21" s="13">
+        <v>20.0</v>
+      </c>
+      <c r="N21" s="13">
+        <f>IF(E16=0, 0, I21/E16)*I25 + IF(E24=0, 0, J21/E24)*J25 + IF(E29=0, 0, K21/E29)*K25 + IF(E30=0, 0, L21/E30)*L25 + IF(E31=0, 0, M21/E31)*M25</f>
+        <v>38.40641407</v>
+      </c>
+      <c r="O21" s="15"/>
+      <c r="P21" s="15"/>
+      <c r="Q21" s="15"/>
+      <c r="R21" s="15"/>
+      <c r="S21" s="15"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="15"/>
+      <c r="B22" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C22" s="20"/>
+      <c r="D22" s="19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E22" s="19">
+        <v>12.0</v>
+      </c>
+      <c r="F22" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G22" s="15"/>
+      <c r="H22" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="I22" s="13">
+        <f>0.6*E16</f>
+        <v>120</v>
+      </c>
+      <c r="J22" s="13">
+        <f>0.6*E24</f>
+        <v>28.8</v>
+      </c>
+      <c r="K22" s="13">
+        <v>15.0</v>
+      </c>
+      <c r="L22" s="13">
+        <v>18.0</v>
+      </c>
+      <c r="M22" s="13">
+        <v>10.0</v>
+      </c>
+      <c r="N22" s="13">
+        <f>IF(E16=0, 0, I22/E16)*I25 + IF(E24=0, 0, J22/E24)*J25 + IF(E29=0, 0, K22/E29)*K25 + IF(E30=0, 0, L22/E30)*L25 + IF(E31=0, 0, M22/E31)*M25</f>
+        <v>28.34555244</v>
+      </c>
+      <c r="O22" s="15"/>
+      <c r="P22" s="15"/>
+      <c r="Q22" s="15"/>
+      <c r="R22" s="15"/>
+      <c r="S22" s="15"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="15"/>
+      <c r="B23" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="20"/>
+      <c r="D23" s="19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E23" s="19">
+        <v>12.0</v>
+      </c>
+      <c r="F23" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G23" s="15"/>
+      <c r="H23" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="I23" s="13">
+        <f>0*E16</f>
+        <v>0</v>
+      </c>
+      <c r="J23" s="13">
+        <f>0*E24</f>
+        <v>0</v>
+      </c>
+      <c r="K23" s="13">
+        <v>0.0</v>
+      </c>
+      <c r="L23" s="13">
+        <v>0.0</v>
+      </c>
+      <c r="M23" s="13">
+        <v>0.0</v>
+      </c>
+      <c r="N23" s="13">
+        <f>IF(E16=0, 0, I23/E16)*I25 + IF(E24=0, 0, J23/E24)*J25 + IF(E29=0, 0, K23/E29)*K25 + IF(E30=0, 0, L23/E30)*L25 + IF(E31=0, 0, M23/E31)*M25</f>
+        <v>0</v>
+      </c>
+      <c r="O23" s="15"/>
+      <c r="P23" s="15"/>
+      <c r="Q23" s="15"/>
+      <c r="R23" s="15"/>
+      <c r="S23" s="15"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="15"/>
+      <c r="B24" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="D24" s="19">
+        <f t="array" ref="D24">SUM(IFERROR(LARGE(D19:D23,{1,2,3,4}),0))</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="19">
+        <f>12*MIN(SUM(F19:F25),COUNT(F19:F23)-1)</f>
+        <v>48</v>
+      </c>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="I24" s="13">
+        <f>D16</f>
+        <v>0</v>
+      </c>
+      <c r="J24" s="13">
+        <f>D24</f>
+        <v>0</v>
+      </c>
+      <c r="K24" s="23" t="str">
+        <f>C29</f>
+        <v/>
+      </c>
+      <c r="L24" s="23" t="str">
+        <f>C30</f>
+        <v/>
+      </c>
+      <c r="M24" s="23" t="str">
+        <f>C31</f>
+        <v/>
+      </c>
+      <c r="N24" s="13">
+        <f>IF(E16=0, 0, I24/E16)*I25 + IF(E24=0, 0, J24/E24)*J25 + IF(E29=0, 0, K24/E29)*K25 + IF(E30=0, 0, L24/E30)*L25 + IF(E31=0, 0, M24/E31)*M25</f>
+        <v>0</v>
+      </c>
+      <c r="O24" s="15"/>
+      <c r="P24" s="15"/>
+      <c r="Q24" s="15"/>
+      <c r="R24" s="15"/>
+      <c r="S24" s="15"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="15"/>
+      <c r="B25" s="15"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="I25" s="13">
+        <v>15.0</v>
+      </c>
+      <c r="J25" s="13">
+        <v>10.0</v>
+      </c>
+      <c r="K25" s="13">
+        <f>75*F29/(F29+F30+F31+2*F32)</f>
+        <v>25</v>
+      </c>
+      <c r="L25" s="13">
+        <f>75*F30/(F29+F30+F31+2*F32)</f>
+        <v>25</v>
+      </c>
+      <c r="M25" s="13">
+        <f>75*F31/(F29+F30+F31+2*F32)</f>
+        <v>25</v>
+      </c>
+      <c r="N25" s="13">
+        <f>SUM(I25:M25)</f>
+        <v>100</v>
+      </c>
+      <c r="O25" s="15"/>
+      <c r="P25" s="15"/>
+      <c r="Q25" s="15"/>
+      <c r="R25" s="15"/>
+      <c r="S25" s="15"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="15"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="15"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="15"/>
+      <c r="L26" s="15"/>
+      <c r="M26" s="15"/>
+      <c r="N26" s="15"/>
+      <c r="O26" s="15"/>
+      <c r="P26" s="15"/>
+      <c r="Q26" s="15"/>
+      <c r="R26" s="15"/>
+      <c r="S26" s="15"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="15"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="15"/>
+      <c r="I27" s="15"/>
+      <c r="J27" s="15"/>
+      <c r="K27" s="15"/>
+      <c r="L27" s="15"/>
+      <c r="M27" s="15"/>
+      <c r="N27" s="15"/>
+      <c r="O27" s="15"/>
+      <c r="P27" s="15"/>
+      <c r="Q27" s="15"/>
+      <c r="R27" s="15"/>
+      <c r="S27" s="15"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="15"/>
+      <c r="B28" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="F28" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+      <c r="I28" s="15"/>
+      <c r="J28" s="15"/>
+      <c r="K28" s="15"/>
+      <c r="L28" s="15"/>
+      <c r="M28" s="15"/>
+      <c r="N28" s="15"/>
+      <c r="O28" s="15"/>
+      <c r="P28" s="15"/>
+      <c r="Q28" s="15"/>
+      <c r="R28" s="15"/>
+      <c r="S28" s="15"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="15"/>
+      <c r="B29" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29" s="20"/>
+      <c r="D29" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="E29" s="19">
+        <v>85.0</v>
+      </c>
+      <c r="F29" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="15"/>
+      <c r="K29" s="15"/>
+      <c r="L29" s="15"/>
+      <c r="M29" s="15"/>
+      <c r="N29" s="15"/>
+      <c r="O29" s="15"/>
+      <c r="P29" s="15"/>
+      <c r="Q29" s="15"/>
+      <c r="R29" s="15"/>
+      <c r="S29" s="15"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="15"/>
+      <c r="B30" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C30" s="20"/>
+      <c r="D30" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="E30" s="19">
+        <v>78.0</v>
+      </c>
+      <c r="F30" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
+      <c r="I30" s="15"/>
+      <c r="J30" s="15"/>
+      <c r="K30" s="15"/>
+      <c r="L30" s="15"/>
+      <c r="M30" s="15"/>
+      <c r="N30" s="15"/>
+      <c r="O30" s="15"/>
+      <c r="P30" s="15"/>
+      <c r="Q30" s="15"/>
+      <c r="R30" s="15"/>
+      <c r="S30" s="15"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="15"/>
+      <c r="B31" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" s="20"/>
+      <c r="D31" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="E31" s="19">
+        <v>79.0</v>
+      </c>
+      <c r="F31" s="19">
+        <v>1.0</v>
+      </c>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+      <c r="I31" s="15"/>
+      <c r="J31" s="15"/>
+      <c r="K31" s="15"/>
+      <c r="L31" s="15"/>
+      <c r="M31" s="15"/>
+      <c r="N31" s="15"/>
+      <c r="O31" s="15"/>
+      <c r="P31" s="15"/>
+      <c r="Q31" s="15"/>
+      <c r="R31" s="15"/>
+      <c r="S31" s="15"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="15"/>
+      <c r="B32" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" s="20"/>
+      <c r="D32" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="F32" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="15"/>
+      <c r="K32" s="15"/>
+      <c r="L32" s="15"/>
+      <c r="M32" s="15"/>
+      <c r="N32" s="15"/>
+      <c r="O32" s="15"/>
+      <c r="P32" s="15"/>
+      <c r="Q32" s="15"/>
+      <c r="R32" s="15"/>
+      <c r="S32" s="15"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="15"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="15"/>
+      <c r="I33" s="15"/>
+      <c r="J33" s="15"/>
+      <c r="K33" s="15"/>
+      <c r="L33" s="15"/>
+      <c r="M33" s="15"/>
+      <c r="N33" s="15"/>
+      <c r="O33" s="15"/>
+      <c r="P33" s="15"/>
+      <c r="Q33" s="15"/>
+      <c r="R33" s="15"/>
+      <c r="S33" s="15"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="15"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
+      <c r="I34" s="15"/>
+      <c r="J34" s="15"/>
+      <c r="K34" s="15"/>
+      <c r="L34" s="15"/>
+      <c r="M34" s="15"/>
+      <c r="N34" s="15"/>
+      <c r="O34" s="15"/>
+      <c r="P34" s="15"/>
+      <c r="Q34" s="15"/>
+      <c r="R34" s="15"/>
+      <c r="S34" s="15"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="15"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="15"/>
+      <c r="K35" s="15"/>
+      <c r="L35" s="15"/>
+      <c r="M35" s="15"/>
+      <c r="N35" s="15"/>
+      <c r="O35" s="15"/>
+      <c r="P35" s="15"/>
+      <c r="Q35" s="15"/>
+      <c r="R35" s="15"/>
+      <c r="S35" s="15"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="15"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+      <c r="I36" s="15"/>
+      <c r="J36" s="15"/>
+      <c r="K36" s="15"/>
+      <c r="L36" s="15"/>
+      <c r="M36" s="15"/>
+      <c r="N36" s="15"/>
+      <c r="O36" s="15"/>
+      <c r="P36" s="15"/>
+      <c r="Q36" s="15"/>
+      <c r="R36" s="15"/>
+      <c r="S36" s="15"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="15"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="15"/>
+      <c r="H37" s="15"/>
+      <c r="I37" s="15"/>
+      <c r="J37" s="15"/>
+      <c r="K37" s="15"/>
+      <c r="L37" s="15"/>
+      <c r="M37" s="15"/>
+      <c r="N37" s="15"/>
+      <c r="O37" s="15"/>
+      <c r="P37" s="15"/>
+      <c r="Q37" s="15"/>
+      <c r="R37" s="15"/>
+      <c r="S37" s="15"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="15"/>
+      <c r="B38" s="15"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="15"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="15"/>
+      <c r="K38" s="15"/>
+      <c r="L38" s="15"/>
+      <c r="M38" s="15"/>
+      <c r="N38" s="15"/>
+      <c r="O38" s="15"/>
+      <c r="P38" s="15"/>
+      <c r="Q38" s="15"/>
+      <c r="R38" s="15"/>
+      <c r="S38" s="15"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="15"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
+      <c r="H39" s="15"/>
+      <c r="I39" s="15"/>
+      <c r="J39" s="15"/>
+      <c r="K39" s="15"/>
+      <c r="L39" s="15"/>
+      <c r="M39" s="15"/>
+      <c r="N39" s="15"/>
+      <c r="O39" s="15"/>
+      <c r="P39" s="15"/>
+      <c r="Q39" s="15"/>
+      <c r="R39" s="15"/>
+      <c r="S39" s="15"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="15"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+      <c r="H40" s="15"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="15"/>
+      <c r="K40" s="15"/>
+      <c r="L40" s="15"/>
+      <c r="M40" s="15"/>
+      <c r="N40" s="15"/>
+      <c r="O40" s="15"/>
+      <c r="P40" s="15"/>
+      <c r="Q40" s="15"/>
+      <c r="R40" s="15"/>
+      <c r="S40" s="15"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="15"/>
+      <c r="B41" s="15"/>
+      <c r="C41" s="16"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+      <c r="H41" s="15"/>
+      <c r="I41" s="15"/>
+      <c r="J41" s="15"/>
+      <c r="K41" s="15"/>
+      <c r="L41" s="15"/>
+      <c r="M41" s="15"/>
+      <c r="N41" s="15"/>
+      <c r="O41" s="15"/>
+      <c r="P41" s="15"/>
+      <c r="Q41" s="15"/>
+      <c r="R41" s="15"/>
+      <c r="S41" s="15"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="15"/>
+      <c r="B42" s="15"/>
+      <c r="C42" s="16"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+      <c r="H42" s="15"/>
+      <c r="I42" s="15"/>
+      <c r="J42" s="15"/>
+      <c r="K42" s="15"/>
+      <c r="L42" s="15"/>
+      <c r="M42" s="15"/>
+      <c r="N42" s="15"/>
+      <c r="O42" s="15"/>
+      <c r="P42" s="15"/>
+      <c r="Q42" s="15"/>
+      <c r="R42" s="15"/>
+      <c r="S42" s="15"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="15"/>
+      <c r="B43" s="15"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="15"/>
+      <c r="G43" s="15"/>
+      <c r="H43" s="15"/>
+      <c r="I43" s="15"/>
+      <c r="J43" s="15"/>
+      <c r="K43" s="15"/>
+      <c r="L43" s="15"/>
+      <c r="M43" s="15"/>
+      <c r="N43" s="15"/>
+      <c r="O43" s="15"/>
+      <c r="P43" s="15"/>
+      <c r="Q43" s="15"/>
+      <c r="R43" s="15"/>
+      <c r="S43" s="15"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>